<commit_message>
Planilha: remove TCPO (catálogo é SINAPI, TCPO fora da fase atual)
Pedro pegou a aba "Referências SINAPI-TCPO" e a decisão registrada é: catálogo =
SINAPI, TCPO fora da fase atual. Alinho o código:

- Motor (main.py): para de rodar o match_tcpo em TODO item — economiza tempo/
  consulta e não popula mais tcpo_matches.
- Planilha (spreadsheet.py): coluna REF sem "TCPO xxx"; aba 3 renomeada de
  "Referências SINAPI-TCPO" → "Referências SINAPI", removido o bloco de renderização
  TCPO + insumos, notas e textos atualizados pra só SINAPI.

Endpoints /api/tcpo/* ficam (mortos, sem UI chamando — mexer neles encostaria na
armadilha de RPC/grant do get_tcpo_details). Exemplo regenerado: 3 abas, ZERO TCPO.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exemplos/quantitativo-exemplo-aiarq.xlsx
+++ b/exemplos/quantitativo-exemplo-aiarq.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo Comparativo" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orçamento" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referências SINAPI-TCPO" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referências SINAPI" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3647,21 +3647,21 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>REFERÊNCIAS SINAPI / TCPO BIM — códigos oficiais por item</t>
+          <t>REFERÊNCIAS SINAPI — códigos oficiais por item</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>SINAPI (Caixa) = referência oficial de preço/quantitativo no Brasil — atualizado mensalmente. TCPO BIM (Pini) = composição técnica com insumos detalhados. Cada item do quantitativo recebe os matches mais próximos pra você buscar preço/composição.</t>
+          <t>SINAPI (Caixa) = referência oficial de preço/quantitativo no Brasil, atualizada mensalmente. Cada item do quantitativo recebe os códigos SINAPI mais próximos pra você buscar o preço/composição.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>AI.arq NÃO entrega preço. Use o código pra consultar o preço atualizado no SINAPI oficial (https://www.caixa.gov.br) ou TCPO BIM. Matches marcados com ~ usaram busca simplificada — confirmar adequação.</t>
+          <t>AI.arq NÃO entrega preço. Use o código pra consultar o preço atualizado no SINAPI oficial (https://www.caixa.gov.br). Matches marcados com ~ usaram busca simplificada — confirmar adequação.</t>
         </is>
       </c>
     </row>
@@ -5489,7 +5489,7 @@
       </c>
       <c r="E85" s="68" t="inlineStr">
         <is>
-          <t>Sem match SINAPI nem TCPO (descrição muito específica) — buscar manualmente em https://www.caixa.gov.br/sinapi</t>
+          <t>Sem match SINAPI (descrição muito específica) — buscar manualmente em https://www.caixa.gov.br/sinapi</t>
         </is>
       </c>
       <c r="F85" s="69" t="n"/>
@@ -5773,7 +5773,7 @@
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
         <is>
-          <t>Como ler: MATCH % indica a similaridade entre a descrição do item e a composição SINAPI/TCPO. Acima de 70% = referência forte. 40-70% = revisar. Abaixo de 30% = candidato fraco, buscar código manualmente em https://www.caixa.gov.br/sinapi.</t>
+          <t>Como ler: MATCH % indica a similaridade entre a descrição do item e a composição SINAPI. Acima de 70% = referência forte. 40-70% = revisar. Abaixo de 30% = candidato fraco, buscar código manualmente em https://www.caixa.gov.br/sinapi.</t>
         </is>
       </c>
     </row>

</xml_diff>